<commit_message>
Blooket som CSV (enligt mallens layout) istället för xlsx
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017mqJrSEX6tzqa8YfkctM6P
</commit_message>
<xml_diff>
--- a/planering/biologi-omrade1/biologi-1-kahoot.xlsx
+++ b/planering/biologi-omrade1/biologi-1-kahoot.xlsx
@@ -1880,17 +1880,17 @@
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
+          <t>bara människokroppen</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>bara djur</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
           <t>bara växter</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>bara människokroppen</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>bara djur</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
@@ -1989,22 +1989,22 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
+          <t>Kontrollgrupp</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Störfaktor</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Beroende variabel</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
           <t>Oberoende variabel</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Störfaktor</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>Beroende variabel</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="inlineStr">
-        <is>
-          <t>Kontrollgrupp</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
@@ -2046,17 +2046,17 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
+          <t>Medelvärde</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Felkälla</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
           <t>Beroende variabel</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Medelvärde</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Felkälla</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
@@ -2108,17 +2108,17 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
+          <t>För att det blir fler deltagare</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
           <t>För att få ett snabbare svar</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>För att slippa mäta</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>För att det blir fler deltagare</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
@@ -2160,17 +2160,17 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
+          <t>Kontroll</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Randomisering</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
           <t>Tendens</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Randomisering</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Kontroll</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
@@ -2217,22 +2217,22 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
+          <t>Medelvärdet</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Datumet</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Enheten</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
           <t>Namnet på forskaren</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>Medelvärdet</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>Enheten</t>
-        </is>
-      </c>
-      <c r="F15" s="14" t="inlineStr">
-        <is>
-          <t>Datumet</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
@@ -2274,17 +2274,17 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
+          <t>Linjediagram</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Kartdiagram</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
           <t>Cirkeldiagram</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Linjediagram</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Kartdiagram</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -2336,12 +2336,12 @@
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
+          <t>Stapeldiagram</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
           <t>Bilddiagram</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Stapeldiagram</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -2502,17 +2502,17 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
+          <t>För att försöket blir billigare</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
           <t>För att få en annan hypotes</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>För att slippa en slutsats</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>För att försöket blir billigare</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -2564,17 +2564,17 @@
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
+          <t>Beroende</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Tendens</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
           <t>Randomisering</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>Beroende</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>Tendens</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
@@ -2616,22 +2616,22 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
+          <t>Hypotes</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Störfaktor</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
           <t>Beroende variabel</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Störfaktor</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>Kontrollgrupp</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Hypotes</t>
         </is>
       </c>
       <c r="G22" s="14" t="n">
@@ -2673,22 +2673,22 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
+          <t>Hooke och Darwin</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
           <t>Mendel och Linné</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Marshall och Warren</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Semmelweis och Pasteur</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Marshall och Warren</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Hooke och Darwin</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
@@ -2735,12 +2735,12 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
+          <t>Att de bär hatt</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
           <t>Att de slutar operera</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>Att de bär hatt</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -2792,17 +2792,17 @@
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
+          <t>Att liv uppstår av sig självt</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Att bakterier är ofarliga</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
           <t>Att luft är farlig</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>Att liv uppstår av sig självt</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Att bakterier är ofarliga</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
@@ -2844,17 +2844,17 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
+          <t>Salmonella enterica</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Helicobacter pylori</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
           <t>Pinus sylvestris</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Helicobacter pylori</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Salmonella enterica</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
@@ -2901,22 +2901,22 @@
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
+          <t>tyckande</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>tendens</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>belägg</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
           <t>pseudovetenskap</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>tyckande</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>belägg</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>tendens</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
@@ -2958,12 +2958,12 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
+          <t>kontrollgrupp</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
           <t>slutsats</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>kontrollgrupp</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
@@ -3020,12 +3020,12 @@
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
+          <t>Äkthet</t>
+        </is>
+      </c>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
           <t>Relevans för din fråga</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>Äkthet</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">

</xml_diff>